<commit_message>
Dejar Solver (solo largos) como método por defecto; Cetes 6.50%
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WmNWFocUbsKFKRbFYkFhb8
</commit_message>
<xml_diff>
--- a/Markowits/Portafolio_Markowitz_Profesor.xlsx
+++ b/Markowits/Portafolio_Markowitz_Profesor.xlsx
@@ -846,10 +846,10 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.0122217948332109</c:v>
+                  <c:v>0.0172079118776168</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.0122217948332109</c:v>
+                  <c:v>0.0172079118776168</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1096,10 +1096,10 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.0122217948332109</c:v>
+                  <c:v>0.0172079118776168</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.0183326922498164</c:v>
+                  <c:v>0.0258118678164251</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1117,7 +1117,7 @@
                   <c:v>0.0817875821358763</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.0901813732038144</c:v>
+                  <c:v>0.0901813732038145</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1379,31 +1379,31 @@
                 <c:formatCode>0.00000000</c:formatCode>
                 <c:ptCount val="9"/>
                 <c:pt idx="0">
-                  <c:v>0.0117644715517125</c:v>
+                  <c:v>0.0134292362819857</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.0118200679176229</c:v>
+                  <c:v>0.0137603941110514</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.0118761254022205</c:v>
+                  <c:v>0.0141262010297019</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.0119326375067375</c:v>
+                  <c:v>0.0145240464794026</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0.0119895978027211</c:v>
+                  <c:v>0.0149513580978967</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0.0120469999327929</c:v>
+                  <c:v>0.0154057133789584</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>0.0121048376113144</c:v>
+                  <c:v>0.0158847678278917</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>0.0121631046249613</c:v>
+                  <c:v>0.0164528228463165</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>0.0122217948332109</c:v>
+                  <c:v>0.0172079118776168</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1415,28 +1415,28 @@
                 <c:formatCode>0.0%</c:formatCode>
                 <c:ptCount val="9"/>
                 <c:pt idx="0">
-                  <c:v>0.065</c:v>
+                  <c:v>0.0649999951295349</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.0670984477669845</c:v>
+                  <c:v>0.0670984488211228</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.069196895533969</c:v>
+                  <c:v>0.0691968808417637</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.0712953433009536</c:v>
+                  <c:v>0.0712953345333515</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0.0733937910679381</c:v>
+                  <c:v>0.0733937303095967</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0.0754922388349227</c:v>
+                  <c:v>0.0754922202455803</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>0.0775906866019072</c:v>
+                  <c:v>0.0775906739371681</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>0.0796891343688918</c:v>
+                  <c:v>0.0796891406688979</c:v>
                 </c:pt>
                 <c:pt idx="8">
                   <c:v>0.0817875821358763</c:v>
@@ -1446,11 +1446,11 @@
           </c:yVal>
           <c:smooth val="0"/>
         </c:ser>
-        <c:axId val="31193797"/>
-        <c:axId val="78387778"/>
+        <c:axId val="8799847"/>
+        <c:axId val="96165564"/>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="31193797"/>
+        <c:axId val="8799847"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1516,12 +1516,12 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="78387778"/>
+        <c:crossAx val="96165564"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="78387778"/>
+        <c:axId val="96165564"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:min val="0.06"/>
@@ -1588,7 +1588,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="31193797"/>
+        <c:crossAx val="8799847"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -21828,7 +21828,7 @@
         <v>27</v>
       </c>
       <c r="I5" s="21" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J5" s="25" t="s">
         <v>28</v>
@@ -21854,7 +21854,7 @@
       </c>
       <c r="D7" s="26" t="n">
         <f aca="false">INDEX(I$48:I$56,MATCH(MAX($K$19:$K$27),$K$19:$K$27,0))</f>
-        <v>0.528379419679543</v>
+        <v>0</v>
       </c>
       <c r="E7" s="23" t="n">
         <f aca="false">AVERAGE(RENDIMIENTOS!$B$3:$B$251)*$I$3</f>
@@ -21878,7 +21878,7 @@
       </c>
       <c r="D8" s="26" t="n">
         <f aca="false">INDEX(J$48:J$56,MATCH(MAX($K$19:$K$27),$K$19:$K$27,0))</f>
-        <v>-0.0639388785210929</v>
+        <v>0</v>
       </c>
       <c r="E8" s="23" t="n">
         <f aca="false">AVERAGE(RENDIMIENTOS!$C$3:$C$251)*$I$3</f>
@@ -21895,7 +21895,7 @@
       </c>
       <c r="D9" s="26" t="n">
         <f aca="false">INDEX(K$48:K$56,MATCH(MAX($K$19:$K$27),$K$19:$K$27,0))</f>
-        <v>0.295536307645177</v>
+        <v>0</v>
       </c>
       <c r="E9" s="23" t="n">
         <f aca="false">AVERAGE(RENDIMIENTOS!$D$3:$D$251)*$I$3</f>
@@ -21910,7 +21910,7 @@
       </c>
       <c r="I9" s="27" t="n">
         <f aca="false">SUMPRODUCT(MMULT(Matriz!$E$31:$L$38,D7:D14),D7:D14)</f>
-        <v>0.000149372268945101</v>
+        <v>0.000296112231187824</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21919,7 +21919,7 @@
       </c>
       <c r="D10" s="26" t="n">
         <f aca="false">INDEX(L$48:L$56,MATCH(MAX($K$19:$K$27),$K$19:$K$27,0))</f>
-        <v>-0.126841528615483</v>
+        <v>0</v>
       </c>
       <c r="E10" s="23" t="n">
         <f aca="false">AVERAGE(RENDIMIENTOS!$E$3:$E$251)*$I$3</f>
@@ -21936,7 +21936,7 @@
       </c>
       <c r="D11" s="26" t="n">
         <f aca="false">INDEX(M$48:M$56,MATCH(MAX($K$19:$K$27),$K$19:$K$27,0))</f>
-        <v>0.108701553907201</v>
+        <v>0</v>
       </c>
       <c r="E11" s="23" t="n">
         <f aca="false">AVERAGE(RENDIMIENTOS!$F$3:$F$251)*$I$3</f>
@@ -21953,7 +21953,7 @@
       </c>
       <c r="D12" s="26" t="n">
         <f aca="false">INDEX(N$48:N$56,MATCH(MAX($K$19:$K$27),$K$19:$K$27,0))</f>
-        <v>0.234019934391866</v>
+        <v>1</v>
       </c>
       <c r="E12" s="23" t="n">
         <f aca="false">AVERAGE(RENDIMIENTOS!$G$3:$G$251)*$I$3</f>
@@ -21968,7 +21968,7 @@
       </c>
       <c r="I12" s="8" t="n">
         <f aca="false">SQRT(I9)</f>
-        <v>0.0122217948332109</v>
+        <v>0.0172079118776168</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21977,7 +21977,7 @@
       </c>
       <c r="D13" s="26" t="n">
         <f aca="false">INDEX(O$48:O$56,MATCH(MAX($K$19:$K$27),$K$19:$K$27,0))</f>
-        <v>0.055145786112025</v>
+        <v>0</v>
       </c>
       <c r="E13" s="23" t="n">
         <f aca="false">AVERAGE(RENDIMIENTOS!$H$3:$H$251)*$I$3</f>
@@ -21994,7 +21994,7 @@
       </c>
       <c r="D14" s="26" t="n">
         <f aca="false">INDEX(P$48:P$56,MATCH(MAX($K$19:$K$27),$K$19:$K$27,0))</f>
-        <v>-0.0310025945992354</v>
+        <v>0</v>
       </c>
       <c r="E14" s="23" t="n">
         <f aca="false">AVERAGE(RENDIMIENTOS!$I$3:$I$251)*$I$3</f>
@@ -22027,7 +22027,7 @@
       </c>
       <c r="F15" s="31" t="n">
         <f aca="false">SUMPRODUCT(D7:D14,F7:F14)</f>
-        <v>0.894254951070821</v>
+        <v>1.14498888583895</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22039,7 +22039,7 @@
       </c>
       <c r="I16" s="9" t="n">
         <f aca="false">+(I7-I14)/I12</f>
-        <v>1.37357747900157</v>
+        <v>0.975573460351852</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -22065,19 +22065,19 @@
       </c>
       <c r="I19" s="34" t="n">
         <f aca="false">SQRT(SUMPRODUCT(MMULT($I48:$P48,Matriz!$E$31:$L$38),$I48:$P48))</f>
-        <v>0.0117644715517125</v>
+        <v>0.0134292362819857</v>
       </c>
       <c r="J19" s="35" t="n">
         <f aca="false">SUMPRODUCT($I48:$P48,$I$46:$P$46)</f>
-        <v>0.065</v>
+        <v>0.0649999951295349</v>
       </c>
       <c r="K19" s="9" t="n">
         <f aca="false">(J19-$I$14)/I19</f>
-        <v>0</v>
+        <v>-3.62676254425688E-007</v>
       </c>
       <c r="L19" s="9" t="n">
         <f aca="false">SUMPRODUCT($I48:$P48,$I$47:$P$47)</f>
-        <v>0.873442556027565</v>
+        <v>1.04813704749361</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22086,19 +22086,19 @@
       </c>
       <c r="I20" s="34" t="n">
         <f aca="false">SQRT(SUMPRODUCT(MMULT($I49:$P49,Matriz!$E$31:$L$38),$I49:$P49))</f>
-        <v>0.0118200679176229</v>
+        <v>0.0137603941110514</v>
       </c>
       <c r="J20" s="35" t="n">
         <f aca="false">SUMPRODUCT($I49:$P49,$I$46:$P$46)</f>
-        <v>0.0670984477669845</v>
+        <v>0.0670984488211228</v>
       </c>
       <c r="K20" s="9" t="n">
         <f aca="false">(J20-$I$14)/I20</f>
-        <v>0.1775326319281</v>
+        <v>0.152499180196985</v>
       </c>
       <c r="L20" s="9" t="n">
         <f aca="false">SUMPRODUCT($I49:$P49,$I$47:$P$47)</f>
-        <v>0.876044105407972</v>
+        <v>1.06773643315597</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22107,19 +22107,19 @@
       </c>
       <c r="I21" s="34" t="n">
         <f aca="false">SQRT(SUMPRODUCT(MMULT($I50:$P50,Matriz!$E$31:$L$38),$I50:$P50))</f>
-        <v>0.0118761254022205</v>
+        <v>0.0141262010297019</v>
       </c>
       <c r="J21" s="35" t="n">
         <f aca="false">SUMPRODUCT($I50:$P50,$I$46:$P$46)</f>
-        <v>0.069196895533969</v>
+        <v>0.0691968808417637</v>
       </c>
       <c r="K21" s="9" t="n">
         <f aca="false">(J21-$I$14)/I21</f>
-        <v>0.35338929085275</v>
+        <v>0.297099045450313</v>
       </c>
       <c r="L21" s="9" t="n">
         <f aca="false">SUMPRODUCT($I50:$P50,$I$47:$P$47)</f>
-        <v>0.878645654788379</v>
+        <v>1.08733525423208</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22128,19 +22128,19 @@
       </c>
       <c r="I22" s="34" t="n">
         <f aca="false">SQRT(SUMPRODUCT(MMULT($I51:$P51,Matriz!$E$31:$L$38),$I51:$P51))</f>
-        <v>0.0119326375067375</v>
+        <v>0.0145240464794026</v>
       </c>
       <c r="J22" s="35" t="n">
         <f aca="false">SUMPRODUCT($I51:$P51,$I$46:$P$46)</f>
-        <v>0.0712953433009536</v>
+        <v>0.0712953345333515</v>
       </c>
       <c r="K22" s="9" t="n">
         <f aca="false">(J22-$I$14)/I22</f>
-        <v>0.527573497259014</v>
+        <v>0.433442191353441</v>
       </c>
       <c r="L22" s="9" t="n">
         <f aca="false">SUMPRODUCT($I51:$P51,$I$47:$P$47)</f>
-        <v>0.881247204168786</v>
+        <v>1.10693463989443</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22149,19 +22149,19 @@
       </c>
       <c r="I23" s="34" t="n">
         <f aca="false">SQRT(SUMPRODUCT(MMULT($I52:$P52,Matriz!$E$31:$L$38),$I52:$P52))</f>
-        <v>0.0119895978027211</v>
+        <v>0.0149513580978967</v>
       </c>
       <c r="J23" s="35" t="n">
         <f aca="false">SUMPRODUCT($I52:$P52,$I$46:$P$46)</f>
-        <v>0.0733937910679381</v>
+        <v>0.0733937303095967</v>
       </c>
       <c r="K23" s="9" t="n">
         <f aca="false">(J23-$I$14)/I23</f>
-        <v>0.700089461385697</v>
+        <v>0.561402533110186</v>
       </c>
       <c r="L23" s="9" t="n">
         <f aca="false">SUMPRODUCT($I52:$P52,$I$47:$P$47)</f>
-        <v>0.883848753549193</v>
+        <v>1.12653273681246</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22170,19 +22170,19 @@
       </c>
       <c r="I24" s="34" t="n">
         <f aca="false">SQRT(SUMPRODUCT(MMULT($I53:$P53,Matriz!$E$31:$L$38),$I53:$P53))</f>
-        <v>0.0120469999327929</v>
+        <v>0.0154057133789584</v>
       </c>
       <c r="J24" s="35" t="n">
         <f aca="false">SUMPRODUCT($I53:$P53,$I$46:$P$46)</f>
-        <v>0.0754922388349227</v>
+        <v>0.0754922202455803</v>
       </c>
       <c r="K24" s="9" t="n">
         <f aca="false">(J24-$I$14)/I24</f>
-        <v>0.870942051419955</v>
+        <v>0.681060330507695</v>
       </c>
       <c r="L24" s="9" t="n">
         <f aca="false">SUMPRODUCT($I53:$P53,$I$47:$P$47)</f>
-        <v>0.8864503029296</v>
+        <v>1.14613284663289</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22191,19 +22191,19 @@
       </c>
       <c r="I25" s="34" t="n">
         <f aca="false">SQRT(SUMPRODUCT(MMULT($I54:$P54,Matriz!$E$31:$L$38),$I54:$P54))</f>
-        <v>0.0121048376113144</v>
+        <v>0.0158847678278917</v>
       </c>
       <c r="J25" s="35" t="n">
         <f aca="false">SUMPRODUCT($I54:$P54,$I$46:$P$46)</f>
-        <v>0.0775906866019072</v>
+        <v>0.0775906739371681</v>
       </c>
       <c r="K25" s="9" t="n">
         <f aca="false">(J25-$I$14)/I25</f>
-        <v>1.04013676235844</v>
+        <v>0.792625619309363</v>
       </c>
       <c r="L25" s="9" t="n">
         <f aca="false">SUMPRODUCT($I54:$P54,$I$47:$P$47)</f>
-        <v>0.889051852310007</v>
+        <v>1.16573223229525</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22212,19 +22212,19 @@
       </c>
       <c r="I26" s="34" t="n">
         <f aca="false">SQRT(SUMPRODUCT(MMULT($I55:$P55,Matriz!$E$31:$L$38),$I55:$P55))</f>
-        <v>0.0121631046249613</v>
+        <v>0.0164528228463165</v>
       </c>
       <c r="J26" s="35" t="n">
         <f aca="false">SUMPRODUCT($I55:$P55,$I$46:$P$46)</f>
-        <v>0.0796891343688918</v>
+        <v>0.0796891406688979</v>
       </c>
       <c r="K26" s="9" t="n">
         <f aca="false">(J26-$I$14)/I26</f>
-        <v>1.20767968555878</v>
+        <v>0.892803673029676</v>
       </c>
       <c r="L26" s="9" t="n">
         <f aca="false">SUMPRODUCT($I55:$P55,$I$47:$P$47)</f>
-        <v>0.891653401690414</v>
+        <v>1.15762542002814</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22233,7 +22233,7 @@
       </c>
       <c r="I27" s="34" t="n">
         <f aca="false">SQRT(SUMPRODUCT(MMULT($I56:$P56,Matriz!$E$31:$L$38),$I56:$P56))</f>
-        <v>0.0122217948332109</v>
+        <v>0.0172079118776168</v>
       </c>
       <c r="J27" s="35" t="n">
         <f aca="false">SUMPRODUCT($I56:$P56,$I$46:$P$46)</f>
@@ -22241,11 +22241,11 @@
       </c>
       <c r="K27" s="9" t="n">
         <f aca="false">(J27-$I$14)/I27</f>
-        <v>1.37357747900157</v>
+        <v>0.975573460351852</v>
       </c>
       <c r="L27" s="9" t="n">
         <f aca="false">SUMPRODUCT($I56:$P56,$I$47:$P$47)</f>
-        <v>0.894254951070821</v>
+        <v>1.14498888583895</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22368,35 +22368,35 @@
       </c>
       <c r="I48" s="39" t="n">
         <f aca="false">IF($I$5=1,I61,I74)</f>
-        <v>0.496295525197577</v>
+        <v>0.284777</v>
       </c>
       <c r="J48" s="39" t="n">
         <f aca="false">IF($I$5=1,J61,J74)</f>
-        <v>-0.0390910816512745</v>
+        <v>0</v>
       </c>
       <c r="K48" s="39" t="n">
         <f aca="false">IF($I$5=1,K61,K74)</f>
-        <v>0.282561702048613</v>
+        <v>0</v>
       </c>
       <c r="L48" s="39" t="n">
         <f aca="false">IF($I$5=1,L61,L74)</f>
-        <v>-0.109633648084208</v>
+        <v>0</v>
       </c>
       <c r="M48" s="39" t="n">
         <f aca="false">IF($I$5=1,M61,M74)</f>
-        <v>0.100888000075036</v>
+        <v>0.159932</v>
       </c>
       <c r="N48" s="39" t="n">
         <f aca="false">IF($I$5=1,N61,N74)</f>
-        <v>0.215930609615409</v>
+        <v>0.555291</v>
       </c>
       <c r="O48" s="39" t="n">
         <f aca="false">IF($I$5=1,O61,O74)</f>
-        <v>0.0582648563133571</v>
+        <v>0</v>
       </c>
       <c r="P48" s="39" t="n">
         <f aca="false">IF($I$5=1,P61,P74)</f>
-        <v>-0.00521596351451034</v>
+        <v>0</v>
       </c>
       <c r="Q48" s="40" t="n">
         <f aca="false">SUM(I48:P48)</f>
@@ -22413,35 +22413,35 @@
       </c>
       <c r="I49" s="39" t="n">
         <f aca="false">IF($I$5=1,I62,I75)</f>
-        <v>0.500306012007823</v>
+        <v>0.2384</v>
       </c>
       <c r="J49" s="39" t="n">
         <f aca="false">IF($I$5=1,J62,J75)</f>
-        <v>-0.0421970562600018</v>
+        <v>0</v>
       </c>
       <c r="K49" s="39" t="n">
         <f aca="false">IF($I$5=1,K62,K75)</f>
-        <v>0.284183527748183</v>
+        <v>0</v>
       </c>
       <c r="L49" s="39" t="n">
         <f aca="false">IF($I$5=1,L62,L75)</f>
-        <v>-0.111784633150617</v>
+        <v>0</v>
       </c>
       <c r="M49" s="39" t="n">
         <f aca="false">IF($I$5=1,M62,M75)</f>
-        <v>0.101864694304057</v>
+        <v>0.160506</v>
       </c>
       <c r="N49" s="39" t="n">
         <f aca="false">IF($I$5=1,N62,N75)</f>
-        <v>0.218191775212466</v>
+        <v>0.601094</v>
       </c>
       <c r="O49" s="39" t="n">
         <f aca="false">IF($I$5=1,O62,O75)</f>
-        <v>0.0578749725381906</v>
+        <v>0</v>
       </c>
       <c r="P49" s="39" t="n">
         <f aca="false">IF($I$5=1,P62,P75)</f>
-        <v>-0.00843929240010092</v>
+        <v>0</v>
       </c>
       <c r="Q49" s="40" t="n">
         <f aca="false">SUM(I49:P49)</f>
@@ -22458,35 +22458,35 @@
       </c>
       <c r="I50" s="39" t="n">
         <f aca="false">IF($I$5=1,I63,I76)</f>
-        <v>0.504316498818069</v>
+        <v>0.192024</v>
       </c>
       <c r="J50" s="39" t="n">
         <f aca="false">IF($I$5=1,J63,J76)</f>
-        <v>-0.0453030308687291</v>
+        <v>0</v>
       </c>
       <c r="K50" s="39" t="n">
         <f aca="false">IF($I$5=1,K63,K76)</f>
-        <v>0.285805353447754</v>
+        <v>0</v>
       </c>
       <c r="L50" s="39" t="n">
         <f aca="false">IF($I$5=1,L63,L76)</f>
-        <v>-0.113935618217027</v>
+        <v>0</v>
       </c>
       <c r="M50" s="39" t="n">
         <f aca="false">IF($I$5=1,M63,M76)</f>
-        <v>0.102841388533077</v>
+        <v>0.161079</v>
       </c>
       <c r="N50" s="39" t="n">
         <f aca="false">IF($I$5=1,N63,N76)</f>
-        <v>0.220452940809523</v>
+        <v>0.646897</v>
       </c>
       <c r="O50" s="39" t="n">
         <f aca="false">IF($I$5=1,O63,O76)</f>
-        <v>0.0574850887630241</v>
+        <v>0</v>
       </c>
       <c r="P50" s="39" t="n">
         <f aca="false">IF($I$5=1,P63,P76)</f>
-        <v>-0.0116626212856916</v>
+        <v>0</v>
       </c>
       <c r="Q50" s="40" t="n">
         <f aca="false">SUM(I50:P50)</f>
@@ -22503,35 +22503,35 @@
       </c>
       <c r="I51" s="39" t="n">
         <f aca="false">IF($I$5=1,I64,I77)</f>
-        <v>0.508326985628314</v>
+        <v>0.145647</v>
       </c>
       <c r="J51" s="39" t="n">
         <f aca="false">IF($I$5=1,J64,J77)</f>
-        <v>-0.0484090054774564</v>
+        <v>0</v>
       </c>
       <c r="K51" s="39" t="n">
         <f aca="false">IF($I$5=1,K64,K77)</f>
-        <v>0.287427179147325</v>
+        <v>0</v>
       </c>
       <c r="L51" s="39" t="n">
         <f aca="false">IF($I$5=1,L64,L77)</f>
-        <v>-0.116086603283436</v>
+        <v>0</v>
       </c>
       <c r="M51" s="39" t="n">
         <f aca="false">IF($I$5=1,M64,M77)</f>
-        <v>0.103818082762098</v>
+        <v>0.161653</v>
       </c>
       <c r="N51" s="39" t="n">
         <f aca="false">IF($I$5=1,N64,N77)</f>
-        <v>0.22271410640658</v>
+        <v>0.6927</v>
       </c>
       <c r="O51" s="39" t="n">
         <f aca="false">IF($I$5=1,O64,O77)</f>
-        <v>0.0570952049878576</v>
+        <v>0</v>
       </c>
       <c r="P51" s="39" t="n">
         <f aca="false">IF($I$5=1,P64,P77)</f>
-        <v>-0.0148859501712823</v>
+        <v>0</v>
       </c>
       <c r="Q51" s="40" t="n">
         <f aca="false">SUM(I51:P51)</f>
@@ -22548,39 +22548,39 @@
       </c>
       <c r="I52" s="39" t="n">
         <f aca="false">IF($I$5=1,I65,I78)</f>
-        <v>0.51233747243856</v>
+        <v>0.09927</v>
       </c>
       <c r="J52" s="39" t="n">
         <f aca="false">IF($I$5=1,J65,J78)</f>
-        <v>-0.0515149800861837</v>
+        <v>0</v>
       </c>
       <c r="K52" s="39" t="n">
         <f aca="false">IF($I$5=1,K65,K78)</f>
-        <v>0.289049004846895</v>
+        <v>0</v>
       </c>
       <c r="L52" s="39" t="n">
         <f aca="false">IF($I$5=1,L65,L78)</f>
-        <v>-0.118237588349846</v>
+        <v>0</v>
       </c>
       <c r="M52" s="39" t="n">
         <f aca="false">IF($I$5=1,M65,M78)</f>
-        <v>0.104794776991119</v>
+        <v>0.162226</v>
       </c>
       <c r="N52" s="39" t="n">
         <f aca="false">IF($I$5=1,N65,N78)</f>
-        <v>0.224975272003637</v>
+        <v>0.738503</v>
       </c>
       <c r="O52" s="39" t="n">
         <f aca="false">IF($I$5=1,O65,O78)</f>
-        <v>0.0567053212126911</v>
+        <v>0</v>
       </c>
       <c r="P52" s="39" t="n">
         <f aca="false">IF($I$5=1,P65,P78)</f>
-        <v>-0.0181092790568729</v>
+        <v>0</v>
       </c>
       <c r="Q52" s="40" t="n">
         <f aca="false">SUM(I52:P52)</f>
-        <v>1</v>
+        <v>0.999999</v>
       </c>
       <c r="R52" s="40" t="n">
         <f aca="false">$I$14+(MAX($E$7:$E$14)-$I$14)*4/8</f>
@@ -22593,35 +22593,35 @@
       </c>
       <c r="I53" s="39" t="n">
         <f aca="false">IF($I$5=1,I66,I79)</f>
-        <v>0.516347959248806</v>
+        <v>0.052894</v>
       </c>
       <c r="J53" s="39" t="n">
         <f aca="false">IF($I$5=1,J66,J79)</f>
-        <v>-0.0546209546949111</v>
+        <v>0</v>
       </c>
       <c r="K53" s="39" t="n">
         <f aca="false">IF($I$5=1,K66,K79)</f>
-        <v>0.290670830546466</v>
+        <v>0</v>
       </c>
       <c r="L53" s="39" t="n">
         <f aca="false">IF($I$5=1,L66,L79)</f>
-        <v>-0.120388573416255</v>
+        <v>0</v>
       </c>
       <c r="M53" s="39" t="n">
         <f aca="false">IF($I$5=1,M66,M79)</f>
-        <v>0.105771471220139</v>
+        <v>0.1628</v>
       </c>
       <c r="N53" s="39" t="n">
         <f aca="false">IF($I$5=1,N66,N79)</f>
-        <v>0.227236437600694</v>
+        <v>0.784306</v>
       </c>
       <c r="O53" s="39" t="n">
         <f aca="false">IF($I$5=1,O66,O79)</f>
-        <v>0.0563154374375245</v>
+        <v>0</v>
       </c>
       <c r="P53" s="39" t="n">
         <f aca="false">IF($I$5=1,P66,P79)</f>
-        <v>-0.0213326079424636</v>
+        <v>0</v>
       </c>
       <c r="Q53" s="40" t="n">
         <f aca="false">SUM(I53:P53)</f>
@@ -22638,35 +22638,35 @@
       </c>
       <c r="I54" s="39" t="n">
         <f aca="false">IF($I$5=1,I67,I80)</f>
-        <v>0.520358446059052</v>
+        <v>0.006517</v>
       </c>
       <c r="J54" s="39" t="n">
         <f aca="false">IF($I$5=1,J67,J80)</f>
-        <v>-0.0577269293036384</v>
+        <v>0</v>
       </c>
       <c r="K54" s="39" t="n">
         <f aca="false">IF($I$5=1,K67,K80)</f>
-        <v>0.292292656246036</v>
+        <v>0</v>
       </c>
       <c r="L54" s="39" t="n">
         <f aca="false">IF($I$5=1,L67,L80)</f>
-        <v>-0.122539558482664</v>
+        <v>0</v>
       </c>
       <c r="M54" s="39" t="n">
         <f aca="false">IF($I$5=1,M67,M80)</f>
-        <v>0.10674816544916</v>
+        <v>0.163374</v>
       </c>
       <c r="N54" s="39" t="n">
         <f aca="false">IF($I$5=1,N67,N80)</f>
-        <v>0.229497603197751</v>
+        <v>0.830109</v>
       </c>
       <c r="O54" s="39" t="n">
         <f aca="false">IF($I$5=1,O67,O80)</f>
-        <v>0.055925553662358</v>
+        <v>0</v>
       </c>
       <c r="P54" s="39" t="n">
         <f aca="false">IF($I$5=1,P67,P80)</f>
-        <v>-0.0245559368280542</v>
+        <v>0</v>
       </c>
       <c r="Q54" s="40" t="n">
         <f aca="false">SUM(I54:P54)</f>
@@ -22683,35 +22683,35 @@
       </c>
       <c r="I55" s="39" t="n">
         <f aca="false">IF($I$5=1,I68,I81)</f>
-        <v>0.524368932869297</v>
+        <v>0</v>
       </c>
       <c r="J55" s="39" t="n">
         <f aca="false">IF($I$5=1,J68,J81)</f>
-        <v>-0.0608329039123656</v>
+        <v>0</v>
       </c>
       <c r="K55" s="39" t="n">
         <f aca="false">IF($I$5=1,K68,K81)</f>
-        <v>0.293914481945607</v>
+        <v>0</v>
       </c>
       <c r="L55" s="39" t="n">
         <f aca="false">IF($I$5=1,L68,L81)</f>
-        <v>-0.124690543549074</v>
+        <v>0</v>
       </c>
       <c r="M55" s="39" t="n">
         <f aca="false">IF($I$5=1,M68,M81)</f>
-        <v>0.10772485967818</v>
+        <v>0.087903</v>
       </c>
       <c r="N55" s="39" t="n">
         <f aca="false">IF($I$5=1,N68,N81)</f>
-        <v>0.231758768794809</v>
+        <v>0.912097</v>
       </c>
       <c r="O55" s="39" t="n">
         <f aca="false">IF($I$5=1,O68,O81)</f>
-        <v>0.0555356698871915</v>
+        <v>0</v>
       </c>
       <c r="P55" s="39" t="n">
         <f aca="false">IF($I$5=1,P68,P81)</f>
-        <v>-0.0277792657136448</v>
+        <v>0</v>
       </c>
       <c r="Q55" s="40" t="n">
         <f aca="false">SUM(I55:P55)</f>
@@ -22728,35 +22728,35 @@
       </c>
       <c r="I56" s="39" t="n">
         <f aca="false">IF($I$5=1,I69,I82)</f>
-        <v>0.528379419679543</v>
+        <v>0</v>
       </c>
       <c r="J56" s="39" t="n">
         <f aca="false">IF($I$5=1,J69,J82)</f>
-        <v>-0.0639388785210929</v>
+        <v>0</v>
       </c>
       <c r="K56" s="39" t="n">
         <f aca="false">IF($I$5=1,K69,K82)</f>
-        <v>0.295536307645177</v>
+        <v>0</v>
       </c>
       <c r="L56" s="39" t="n">
         <f aca="false">IF($I$5=1,L69,L82)</f>
-        <v>-0.126841528615483</v>
+        <v>0</v>
       </c>
       <c r="M56" s="39" t="n">
         <f aca="false">IF($I$5=1,M69,M82)</f>
-        <v>0.108701553907201</v>
+        <v>0</v>
       </c>
       <c r="N56" s="39" t="n">
         <f aca="false">IF($I$5=1,N69,N82)</f>
-        <v>0.234019934391866</v>
+        <v>1</v>
       </c>
       <c r="O56" s="39" t="n">
         <f aca="false">IF($I$5=1,O69,O82)</f>
-        <v>0.055145786112025</v>
+        <v>0</v>
       </c>
       <c r="P56" s="39" t="n">
         <f aca="false">IF($I$5=1,P69,P82)</f>
-        <v>-0.0310025945992354</v>
+        <v>0</v>
       </c>
       <c r="Q56" s="40" t="n">
         <f aca="false">SUM(I56:P56)</f>
@@ -23648,7 +23648,7 @@
     <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H91" s="8" t="n">
         <f aca="false">$I$12</f>
-        <v>0.0122217948332109</v>
+        <v>0.0172079118776168</v>
       </c>
       <c r="I91" s="23" t="n">
         <f aca="false">$I$7</f>
@@ -23667,7 +23667,7 @@
       </c>
       <c r="N91" s="8" t="n">
         <f aca="false">MAX($I$19:$I$27)</f>
-        <v>0.0122217948332109</v>
+        <v>0.0172079118776168</v>
       </c>
       <c r="O91" s="23" t="n">
         <f aca="false">MAX($J$19:$J$27)</f>
@@ -23677,11 +23677,11 @@
     <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H92" s="8" t="n">
         <f aca="false">1.5*$I$12</f>
-        <v>0.0183326922498164</v>
+        <v>0.0258118678164251</v>
       </c>
       <c r="I92" s="23" t="n">
         <f aca="false">$I$14+1.5*($I$7-$I$14)</f>
-        <v>0.0901813732038144</v>
+        <v>0.0901813732038145</v>
       </c>
       <c r="K92" s="43" t="n">
         <v>1.5</v>
@@ -23696,7 +23696,7 @@
       </c>
       <c r="N92" s="8" t="n">
         <f aca="false">MAX($I$19:$I$27)</f>
-        <v>0.0122217948332109</v>
+        <v>0.0172079118776168</v>
       </c>
       <c r="O92" s="23" t="n">
         <f aca="false">$I$14</f>

</xml_diff>